<commit_message>
PAUSED (task156): loop 3 at stage 4, every free gate green and the leak reader clean, the judge thread running
target.zip f17b387d: checks 110, verify agreeing (32 FTE: 5 2 6 4 4 2 4 3 2), two byte-identical
builds, figures_check 112/0, precut 52/0, voice-check PASS, leak.py REVIEW with no LEAK (no file
describes the data), heart WARN, surface with no hard tell (task157, task452 and task265
differentiated on the card). The isolated leak reader found no decisive-step sentence, no ranking
file and no helper-only file, and classed the decision analytical. Resume: the judge thread's
verdict, the pass-3 report, then RESHIPPED.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142Jt4Mt622iBfGoK24ivCU
</commit_message>
<xml_diff>
--- a/task156/golden/moderation_pool_2027.xlsx
+++ b/task156/golden/moderation_pool_2027.xlsx
@@ -25,9 +25,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="132">
-  <si>
-    <t>The nine sites need 35 paid moderator FTE in 2027, 9 above finance's envelope</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="142">
+  <si>
+    <t>The nine sites need 32 paid moderator FTE in 2027, 6 above finance's envelope</t>
   </si>
   <si>
     <t>Need as the charter defines it (section 4): the hours the paid team will spend in 2027 on each site's moderator flags and on the community review items no volunteer has reviewed 72 hours after they entered the inbox, each at the 2027 handle-time standard. One FTE is 1,600 hours; each site to the nearest whole FTE; the request is the sum of the nine.</t>
@@ -102,28 +102,58 @@
     <t>Pool funded for 2026 (FTE)</t>
   </si>
   <si>
-    <t>Every site's reviewer pool is losing about 2 per cent a month, with almost no new reviewers</t>
-  </si>
-  <si>
-    <t>Active reviewers made at least one review in the month (reviewer roster). Each pool is carried forward month by month at its own lapse rate, with the new reviewers it has been getting; every reviewer at about 40 reviews a month, the pace reviewers keep when the inbox outruns them.</t>
+    <t>The 10,607 reviewers active in September 2026 average about 8,800 a month in 2027: the newest leave fastest</t>
+  </si>
+  <si>
+    <t>Active reviewers made at least one review in the month (reviewer roster). Review access has been by invitation only since 1 September 2026 (operations handbook), so a site's pool now only shrinks. Each reviewer is carried forward on the monthly stop rate the roster shows at their tenure (months since access was granted), every reviewer at about 40 reviews a month, the pace reviewers keep when the inbox outruns them.</t>
   </si>
   <si>
     <t>Active reviewers, September 2026</t>
   </si>
   <si>
-    <t>Lapsing a month, September 2024 to August 2026</t>
-  </si>
-  <si>
-    <t>New reviewers a month, October 2025 to September 2026</t>
-  </si>
-  <si>
-    <t>Active reviewers, December 2027</t>
+    <t>Of whom granted access in the previous twelve months</t>
+  </si>
+  <si>
+    <t>Active reviewers expected, June 2027</t>
+  </si>
+  <si>
+    <t>Active reviewers expected, December 2027</t>
   </si>
   <si>
     <t>Months short of the inbox, October 2026 to December 2027</t>
   </si>
   <si>
-    <t>New reviewers across the network: 2,871 in 2024, 70 from January 2025 to September 2026.</t>
+    <t>Monthly stop rate by tenure, all nine sites, January 2024 to August 2026</t>
+  </si>
+  <si>
+    <t>Tenure</t>
+  </si>
+  <si>
+    <t>Reviewer-months at risk</t>
+  </si>
+  <si>
+    <t>Stops</t>
+  </si>
+  <si>
+    <t>Stop rate a month</t>
+  </si>
+  <si>
+    <t>First year</t>
+  </si>
+  <si>
+    <t>Second year</t>
+  </si>
+  <si>
+    <t>Third year</t>
+  </si>
+  <si>
+    <t>Fourth year</t>
+  </si>
+  <si>
+    <t>Fifth year and later</t>
+  </si>
+  <si>
+    <t>A reviewer is at risk from the first month the platform's record (January 2024 on) shows them active to their last review; a stop is the last review of a reviewer whose access lapsed. The projection uses the rate for each month of tenure; the bands summarise it.</t>
   </si>
   <si>
     <t>Moderator flags answered within 24 hours, July to September 2026: Security, Embedded &amp; Hardware and Scientific Computing answered fewer</t>
@@ -168,7 +198,7 @@
     <t>Paid review hours by month and site, January 2024 to December 2027 (the deck's chart)</t>
   </si>
   <si>
-    <t>Paid review hours as the operations notes define them: each moderator flag a paid moderator handled and each community item routed to the team, at the handle-time standard in force for its year (close votes 5.0 minutes to December 2026, 2.0 from January 2027), in the month the flag was raised or the item entered the inbox, UTC. Actual to September 2026; forecast from October 2026 on the question plan and its outlook.</t>
+    <t>Paid review hours as the operations handbook defines them: each moderator flag a paid moderator handled and each community item routed to the team, at the handle-time standard in force for its year (close votes 5.0 minutes to December 2026, 2.0 from January 2027), in the month the flag was raised or the item entered the inbox, UTC. Actual to September 2026; forecast from October 2026 on the question plan and its outlook.</t>
   </si>
   <si>
     <t>Month</t>
@@ -372,13 +402,13 @@
     <t>Reviewer pace</t>
   </si>
   <si>
-    <t>About 40 reviews a month per active reviewer: volunteer reviews over active reviewers in the 89 site-months, 2021 to September 2026, in which more than 5 per cent of the items entering the inbox reached the paid team (the old review system's workbook to 2023; the inbox export and the reviewer roster from 2024). When the inbox runs dry, reviewers review only what arrives, so those months show the work, not the pace.</t>
+    <t>About 40 reviews a month per active reviewer: volunteer reviews over active reviewers in the 402 site-months, 2021 to September 2026, in which more than 5 per cent of the items entering the inbox reached the paid team (the old review system's workbook to 2023; the inbox export and the reviewer roster from 2024). When the inbox runs dry, reviewers review only what arrives, so those months show the work, not the pace.</t>
   </si>
   <si>
     <t>Reviewer pools</t>
   </si>
   <si>
-    <t>Each site's active reviewers in September 2026, carried forward month by month less the share that lapses each month (lapses over active reviewer-months, September 2024 to August 2026, the last full month of lapses the roster shows; about 2 per cent on every site) plus the new reviewers a month of the last twelve months. Almost no member has been granted review access since late 2024.</t>
+    <t>Review access has been by invitation only since 1 September 2026 and nobody was invited in September, so the 2027 pool is the September 2026 pool, shrinking. Reviewers stop at very different rates by tenure: about 9 per cent a month in their first year, under one per cent from their fourth (the stop-rate table on the Reviewer pools sheet, every reviewer counted from the month the roster first shows them active, so those granted before 2024 enter at their tenure then). Each reviewer is carried on the rate for their own tenure month by month. The pool's overall lapse rate of the last two years, about 3 per cent a month, was the rate of a pool still taking in newcomers; carried into a closed pool it would overstate 2027's losses.</t>
   </si>
   <si>
     <t>Items reaching the team</t>
@@ -396,7 +426,7 @@
     <t>Where cover runs out</t>
   </si>
   <si>
-    <t>Data &amp; ML, Databases, Infrastructure &amp; DevOps and Game Development have sent the paid team only the items no volunteer picks up since January 2024; at the pace and lapse rate above, their pools fall short of the inbox from October 2026 and in most months of 2027. Security, Embedded &amp; Hardware and Scientific Computing are short already. Frontend &amp; Web and Mobile Apps stay covered through 2027.</t>
+    <t>Data &amp; ML, Databases, Infrastructure &amp; DevOps and Game Development have sent the paid team only the items no volunteer picks up since January 2024; at the pace and the pools above, they fall short of the inbox from October 2026 and in most months of 2027. Security, Embedded &amp; Hardware and Scientific Computing are short already. Frontend &amp; Web and Mobile Apps stay covered through 2027.</t>
   </si>
   <si>
     <t>Flag response</t>
@@ -414,13 +444,13 @@
     <t>Questions vs 2022</t>
   </si>
   <si>
-    <t>The old statistics job counted a question on every site it was posted to, so a moved question counted on its first site in the month it was asked and again on its new site in the month it moved (posts warehouse notes). Comparisons are on the warehouse's basis: the migration log puts each moved question on the site it moved to, in the month it was asked, once.</t>
+    <t>The old statistics job counted a question on every site it was posted to, so a moved question counted on its first site in the month it was asked and again on its new site in the month it moved (question count standard). Comparisons are on the warehouse's basis: the migration log puts each moved question on the site it moved to, in the month it was asked, once.</t>
   </si>
   <si>
     <t>Paid review hours</t>
   </si>
   <si>
-    <t>The deck's chart, as the operations notes define them: each moderator flag a paid moderator handled and each community item routed to the team, at the standard in force for its year, in the month the flag was raised or the item entered the inbox (UTC); not the hours worked on the WFM lines.</t>
+    <t>The deck's chart, as the operations handbook defines them: each moderator flag a paid moderator handled and each community item routed to the team, at the standard in force for its year, in the month the flag was raised or the item entered the inbox (UTC); not the hours worked on the WFM lines.</t>
   </si>
 </sst>
 </file>
@@ -494,7 +524,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -508,10 +538,6 @@
     <xf numFmtId="3" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="10" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -890,13 +916,13 @@
         <v>998313</v>
       </c>
       <c r="E6" s="4">
-        <v>1285905</v>
+        <v>1396577</v>
       </c>
       <c r="F6" s="4">
-        <v>5739</v>
+        <v>5785</v>
       </c>
       <c r="G6" s="4">
-        <v>8520</v>
+        <v>8522</v>
       </c>
       <c r="H6">
         <v>5</v>
@@ -916,13 +942,13 @@
         <v>382132</v>
       </c>
       <c r="E7" s="4">
-        <v>488543</v>
+        <v>496047</v>
       </c>
       <c r="F7" s="4">
-        <v>2197</v>
+        <v>2214</v>
       </c>
       <c r="G7" s="4">
-        <v>2958</v>
+        <v>2959</v>
       </c>
       <c r="H7">
         <v>2</v>
@@ -942,16 +968,16 @@
         <v>770772</v>
       </c>
       <c r="E8" s="4">
-        <v>664492</v>
+        <v>690967</v>
       </c>
       <c r="F8" s="4">
-        <v>106364</v>
+        <v>81850</v>
       </c>
       <c r="G8" s="4">
-        <v>11236</v>
+        <v>9990</v>
       </c>
       <c r="H8">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -968,16 +994,16 @@
         <v>631425</v>
       </c>
       <c r="E9" s="4">
-        <v>561562</v>
+        <v>602575</v>
       </c>
       <c r="F9" s="4">
-        <v>71348</v>
+        <v>42034</v>
       </c>
       <c r="G9" s="4">
-        <v>8115</v>
+        <v>6636</v>
       </c>
       <c r="H9">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -994,16 +1020,16 @@
         <v>536217</v>
       </c>
       <c r="E10" s="4">
-        <v>477806</v>
+        <v>509964</v>
       </c>
       <c r="F10" s="4">
-        <v>59760</v>
+        <v>36777</v>
       </c>
       <c r="G10" s="4">
-        <v>7758</v>
+        <v>6607</v>
       </c>
       <c r="H10">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -1020,13 +1046,13 @@
         <v>207213</v>
       </c>
       <c r="E11" s="4">
-        <v>177200</v>
+        <v>178647</v>
       </c>
       <c r="F11" s="4">
-        <v>30013</v>
+        <v>28578</v>
       </c>
       <c r="G11" s="4">
-        <v>3265</v>
+        <v>3193</v>
       </c>
       <c r="H11">
         <v>2</v>
@@ -1046,13 +1072,13 @@
         <v>262946</v>
       </c>
       <c r="E12" s="4">
-        <v>176706</v>
+        <v>172459</v>
       </c>
       <c r="F12" s="4">
-        <v>86240</v>
+        <v>90486</v>
       </c>
       <c r="G12" s="4">
-        <v>6181</v>
+        <v>6394</v>
       </c>
       <c r="H12">
         <v>4</v>
@@ -1072,13 +1098,13 @@
         <v>177048</v>
       </c>
       <c r="E13" s="4">
-        <v>105273</v>
+        <v>105796</v>
       </c>
       <c r="F13" s="4">
-        <v>71775</v>
+        <v>71252</v>
       </c>
       <c r="G13" s="4">
-        <v>4828</v>
+        <v>4802</v>
       </c>
       <c r="H13">
         <v>3</v>
@@ -1098,13 +1124,13 @@
         <v>121197</v>
       </c>
       <c r="E14" s="4">
-        <v>76371</v>
+        <v>74262</v>
       </c>
       <c r="F14" s="4">
-        <v>44826</v>
+        <v>46935</v>
       </c>
       <c r="G14" s="4">
-        <v>3094</v>
+        <v>3202</v>
       </c>
       <c r="H14">
         <v>2</v>
@@ -1124,16 +1150,16 @@
         <v>4087264</v>
       </c>
       <c r="E15" s="6">
-        <v>4013857</v>
+        <v>4227295</v>
       </c>
       <c r="F15" s="6">
-        <v>478261</v>
+        <v>405913</v>
       </c>
       <c r="G15" s="6">
-        <v>55955</v>
+        <v>52304</v>
       </c>
       <c r="H15" s="5">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
@@ -1141,7 +1167,7 @@
         <v>21</v>
       </c>
       <c r="H17" s="7">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
@@ -1157,7 +1183,7 @@
         <v>23</v>
       </c>
       <c r="H19" s="7">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
@@ -1184,13 +1210,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC28450C-345D-5267-9D00-367C9A38FD95}">
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.7109375" customWidth="1"/>
     <col min="2" max="2" width="14.7109375" customWidth="1"/>
-    <col min="3" max="3" width="16.7109375" customWidth="1"/>
-    <col min="4" max="4" width="17.7109375" customWidth="1"/>
+    <col min="3" max="3" width="17.7109375" customWidth="1"/>
+    <col min="4" max="4" width="14.7109375" customWidth="1"/>
     <col min="5" max="5" width="14.7109375" customWidth="1"/>
     <col min="6" max="6" width="17.7109375" customWidth="1"/>
   </cols>
@@ -1200,7 +1226,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>26</v>
       </c>
@@ -1230,16 +1256,16 @@
         <v>11</v>
       </c>
       <c r="B5" s="4">
-        <v>3246</v>
-      </c>
-      <c r="C5" s="9">
-        <v>0.02039593848812774</v>
-      </c>
-      <c r="D5" s="10">
-        <v>0.33</v>
+        <v>3412</v>
+      </c>
+      <c r="C5" s="4">
+        <v>526</v>
+      </c>
+      <c r="D5" s="4">
+        <v>2912</v>
       </c>
       <c r="E5" s="4">
-        <v>2387</v>
+        <v>2733</v>
       </c>
       <c r="F5">
         <v>0</v>
@@ -1250,16 +1276,16 @@
         <v>12</v>
       </c>
       <c r="B6" s="4">
-        <v>1230</v>
-      </c>
-      <c r="C6" s="9">
-        <v>0.02030443621956941</v>
-      </c>
-      <c r="D6" s="10">
-        <v>0.33</v>
+        <v>1205</v>
+      </c>
+      <c r="C6" s="4">
+        <v>174</v>
+      </c>
+      <c r="D6" s="4">
+        <v>1034</v>
       </c>
       <c r="E6" s="4">
-        <v>909</v>
+        <v>973</v>
       </c>
       <c r="F6">
         <v>0</v>
@@ -1270,19 +1296,19 @@
         <v>13</v>
       </c>
       <c r="B7" s="4">
-        <v>1679</v>
-      </c>
-      <c r="C7" s="9">
-        <v>0.02049483363351976</v>
-      </c>
-      <c r="D7" s="10">
-        <v>0.17</v>
+        <v>1784</v>
+      </c>
+      <c r="C7" s="4">
+        <v>426</v>
+      </c>
+      <c r="D7" s="4">
+        <v>1439</v>
       </c>
       <c r="E7" s="4">
-        <v>1233</v>
+        <v>1329</v>
       </c>
       <c r="F7">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -1290,19 +1316,19 @@
         <v>14</v>
       </c>
       <c r="B8" s="4">
-        <v>1419</v>
-      </c>
-      <c r="C8" s="9">
-        <v>0.02058578160582625</v>
-      </c>
-      <c r="D8" s="10">
-        <v>0.25</v>
+        <v>1530</v>
+      </c>
+      <c r="C8" s="4">
+        <v>324</v>
+      </c>
+      <c r="D8" s="4">
+        <v>1255</v>
       </c>
       <c r="E8" s="4">
-        <v>1042</v>
+        <v>1165</v>
       </c>
       <c r="F8">
-        <v>13</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -1310,19 +1336,19 @@
         <v>15</v>
       </c>
       <c r="B9" s="4">
-        <v>1202</v>
-      </c>
-      <c r="C9" s="9">
-        <v>0.02060867481428229</v>
-      </c>
-      <c r="D9" s="10">
-        <v>0.75</v>
+        <v>1287</v>
+      </c>
+      <c r="C9" s="4">
+        <v>262</v>
+      </c>
+      <c r="D9" s="4">
+        <v>1063</v>
       </c>
       <c r="E9" s="4">
-        <v>889</v>
+        <v>988</v>
       </c>
       <c r="F9">
-        <v>13</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -1330,16 +1356,16 @@
         <v>16</v>
       </c>
       <c r="B10" s="4">
-        <v>449</v>
-      </c>
-      <c r="C10" s="9">
-        <v>0.02068281626292676</v>
-      </c>
-      <c r="D10" s="10">
-        <v>0</v>
+        <v>451</v>
+      </c>
+      <c r="C10" s="4">
+        <v>87</v>
+      </c>
+      <c r="D10" s="4">
+        <v>372</v>
       </c>
       <c r="E10" s="4">
-        <v>328</v>
+        <v>346</v>
       </c>
       <c r="F10">
         <v>14</v>
@@ -1350,16 +1376,16 @@
         <v>17</v>
       </c>
       <c r="B11" s="4">
-        <v>446</v>
-      </c>
-      <c r="C11" s="9">
-        <v>0.02026881334004169</v>
-      </c>
-      <c r="D11" s="10">
-        <v>0</v>
+        <v>451</v>
+      </c>
+      <c r="C11" s="4">
+        <v>118</v>
+      </c>
+      <c r="D11" s="4">
+        <v>359</v>
       </c>
       <c r="E11" s="4">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="F11">
         <v>15</v>
@@ -1370,16 +1396,16 @@
         <v>18</v>
       </c>
       <c r="B12" s="4">
-        <v>266</v>
-      </c>
-      <c r="C12" s="9">
-        <v>0.02038613742654995</v>
-      </c>
-      <c r="D12" s="10">
-        <v>0</v>
+        <v>288</v>
+      </c>
+      <c r="C12" s="4">
+        <v>91</v>
+      </c>
+      <c r="D12" s="4">
+        <v>220</v>
       </c>
       <c r="E12" s="4">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="F12">
         <v>15</v>
@@ -1390,13 +1416,13 @@
         <v>19</v>
       </c>
       <c r="B13" s="4">
-        <v>194</v>
-      </c>
-      <c r="C13" s="9">
-        <v>0.02094926350245499</v>
-      </c>
-      <c r="D13" s="10">
-        <v>0</v>
+        <v>199</v>
+      </c>
+      <c r="C13" s="4">
+        <v>58</v>
+      </c>
+      <c r="D13" s="4">
+        <v>155</v>
       </c>
       <c r="E13" s="4">
         <v>141</v>
@@ -1410,28 +1436,117 @@
         <v>20</v>
       </c>
       <c r="B14" s="6">
-        <v>10131</v>
-      </c>
-      <c r="C14" s="11">
-        <v>0.02047060973803544</v>
-      </c>
-      <c r="D14" s="12">
-        <v>1.83</v>
+        <v>10607</v>
+      </c>
+      <c r="C14" s="6">
+        <v>2066</v>
+      </c>
+      <c r="D14" s="6">
+        <v>8810</v>
       </c>
       <c r="E14" s="6">
-        <v>7453</v>
+        <v>8205</v>
       </c>
       <c r="F14" s="5"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+      <c r="A16" s="7" t="s">
         <v>32</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>37</v>
+      </c>
+      <c r="B18" s="4">
+        <v>83454</v>
+      </c>
+      <c r="C18" s="4">
+        <v>7569</v>
+      </c>
+      <c r="D18" s="9">
+        <v>9.1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>38</v>
+      </c>
+      <c r="B19" s="4">
+        <v>40676</v>
+      </c>
+      <c r="C19" s="4">
+        <v>2111</v>
+      </c>
+      <c r="D19" s="9">
+        <v>5.2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>39</v>
+      </c>
+      <c r="B20" s="4">
+        <v>32278</v>
+      </c>
+      <c r="C20" s="4">
+        <v>721</v>
+      </c>
+      <c r="D20" s="9">
+        <v>2.2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>40</v>
+      </c>
+      <c r="B21" s="4">
+        <v>30397</v>
+      </c>
+      <c r="C21" s="4">
+        <v>279</v>
+      </c>
+      <c r="D21" s="9">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22" s="4">
+        <v>170542</v>
+      </c>
+      <c r="C22" s="4">
+        <v>909</v>
+      </c>
+      <c r="D22" s="9">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A24:F24"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A16:F16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1450,12 +1565,12 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -1463,26 +1578,26 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="13">
+      <c r="B5" s="9">
         <v>97.90000000000001</v>
       </c>
-      <c r="C5" s="13">
+      <c r="C5" s="9">
         <v>97</v>
       </c>
-      <c r="D5" s="13">
+      <c r="D5" s="9">
         <v>97.09999999999999</v>
       </c>
     </row>
@@ -1490,13 +1605,13 @@
       <c r="A6" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="13">
+      <c r="B6" s="9">
         <v>97.2</v>
       </c>
-      <c r="C6" s="13">
+      <c r="C6" s="9">
         <v>96.40000000000001</v>
       </c>
-      <c r="D6" s="13">
+      <c r="D6" s="9">
         <v>96.3</v>
       </c>
     </row>
@@ -1504,13 +1619,13 @@
       <c r="A7" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="13">
+      <c r="B7" s="9">
         <v>97.8</v>
       </c>
-      <c r="C7" s="13">
+      <c r="C7" s="9">
         <v>97.3</v>
       </c>
-      <c r="D7" s="13">
+      <c r="D7" s="9">
         <v>97.40000000000001</v>
       </c>
     </row>
@@ -1518,13 +1633,13 @@
       <c r="A8" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="13">
+      <c r="B8" s="9">
         <v>97.09999999999999</v>
       </c>
-      <c r="C8" s="13">
+      <c r="C8" s="9">
         <v>97.5</v>
       </c>
-      <c r="D8" s="13">
+      <c r="D8" s="9">
         <v>96.40000000000001</v>
       </c>
     </row>
@@ -1532,13 +1647,13 @@
       <c r="A9" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="13">
+      <c r="B9" s="9">
         <v>98</v>
       </c>
-      <c r="C9" s="13">
+      <c r="C9" s="9">
         <v>96.8</v>
       </c>
-      <c r="D9" s="13">
+      <c r="D9" s="9">
         <v>96.7</v>
       </c>
     </row>
@@ -1546,13 +1661,13 @@
       <c r="A10" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="13">
+      <c r="B10" s="9">
         <v>97.59999999999999</v>
       </c>
-      <c r="C10" s="13">
+      <c r="C10" s="9">
         <v>96.8</v>
       </c>
-      <c r="D10" s="13">
+      <c r="D10" s="9">
         <v>96.2</v>
       </c>
     </row>
@@ -1560,13 +1675,13 @@
       <c r="A11" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="13">
+      <c r="B11" s="9">
         <v>91.8</v>
       </c>
-      <c r="C11" s="13">
+      <c r="C11" s="9">
         <v>89.3</v>
       </c>
-      <c r="D11" s="13">
+      <c r="D11" s="9">
         <v>88.09999999999999</v>
       </c>
     </row>
@@ -1574,13 +1689,13 @@
       <c r="A12" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="13">
+      <c r="B12" s="9">
         <v>91.40000000000001</v>
       </c>
-      <c r="C12" s="13">
+      <c r="C12" s="9">
         <v>87.7</v>
       </c>
-      <c r="D12" s="13">
+      <c r="D12" s="9">
         <v>87.09999999999999</v>
       </c>
     </row>
@@ -1588,13 +1703,13 @@
       <c r="A13" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="13">
+      <c r="B13" s="9">
         <v>85.59999999999999</v>
       </c>
-      <c r="C13" s="13">
+      <c r="C13" s="9">
         <v>90</v>
       </c>
-      <c r="D13" s="13">
+      <c r="D13" s="9">
         <v>81.40000000000001</v>
       </c>
     </row>
@@ -1619,12 +1734,12 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -1632,13 +1747,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -1786,12 +1901,12 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1799,14 +1914,14 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="13">
+      <c r="B5" s="9">
         <v>39.7</v>
       </c>
     </row>
@@ -1814,7 +1929,7 @@
       <c r="A6" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="13">
+      <c r="B6" s="9">
         <v>42.1</v>
       </c>
     </row>
@@ -1822,7 +1937,7 @@
       <c r="A7" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="13">
+      <c r="B7" s="9">
         <v>55.5</v>
       </c>
     </row>
@@ -1830,7 +1945,7 @@
       <c r="A8" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="13">
+      <c r="B8" s="9">
         <v>58.4</v>
       </c>
     </row>
@@ -1838,7 +1953,7 @@
       <c r="A9" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="13">
+      <c r="B9" s="9">
         <v>60.2</v>
       </c>
     </row>
@@ -1846,7 +1961,7 @@
       <c r="A10" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="13">
+      <c r="B10" s="9">
         <v>53.8</v>
       </c>
     </row>
@@ -1854,7 +1969,7 @@
       <c r="A11" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="13">
+      <c r="B11" s="9">
         <v>72</v>
       </c>
     </row>
@@ -1862,7 +1977,7 @@
       <c r="A12" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="13">
+      <c r="B12" s="9">
         <v>76</v>
       </c>
     </row>
@@ -1870,7 +1985,7 @@
       <c r="A13" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="13">
+      <c r="B13" s="9">
         <v>76.8</v>
       </c>
     </row>
@@ -1904,20 +2019,20 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>11</v>
@@ -1950,15 +2065,15 @@
         <v>20</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="B5" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C5" s="4">
         <v>903</v>
@@ -1976,19 +2091,19 @@
         <v>477</v>
       </c>
       <c r="H5" s="4">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="I5" s="4">
-        <v>181</v>
+        <v>556</v>
       </c>
       <c r="J5" s="4">
-        <v>115</v>
+        <v>417</v>
       </c>
       <c r="K5" s="4">
-        <v>74</v>
+        <v>227</v>
       </c>
       <c r="L5" s="4">
-        <v>3263</v>
+        <v>4096</v>
       </c>
       <c r="M5" s="4">
         <v>3467</v>
@@ -1996,10 +2111,10 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="B6" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C6" s="4">
         <v>922</v>
@@ -2017,19 +2132,19 @@
         <v>495</v>
       </c>
       <c r="H6" s="4">
-        <v>192</v>
+        <v>292</v>
       </c>
       <c r="I6" s="4">
-        <v>178</v>
+        <v>634</v>
       </c>
       <c r="J6" s="4">
-        <v>119</v>
+        <v>392</v>
       </c>
       <c r="K6" s="4">
-        <v>74</v>
+        <v>294</v>
       </c>
       <c r="L6" s="4">
-        <v>3367</v>
+        <v>4415</v>
       </c>
       <c r="M6" s="4">
         <v>3467</v>
@@ -2037,10 +2152,10 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="B7" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C7" s="4">
         <v>942</v>
@@ -2058,19 +2173,19 @@
         <v>506</v>
       </c>
       <c r="H7" s="4">
-        <v>180</v>
+        <v>349</v>
       </c>
       <c r="I7" s="4">
-        <v>190</v>
+        <v>654</v>
       </c>
       <c r="J7" s="4">
-        <v>124</v>
+        <v>482</v>
       </c>
       <c r="K7" s="4">
-        <v>74</v>
+        <v>328</v>
       </c>
       <c r="L7" s="4">
-        <v>3468</v>
+        <v>4713</v>
       </c>
       <c r="M7" s="4">
         <v>3467</v>
@@ -2078,10 +2193,10 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="B8" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C8" s="4">
         <v>905</v>
@@ -2099,19 +2214,19 @@
         <v>482</v>
       </c>
       <c r="H8" s="4">
-        <v>181</v>
+        <v>198</v>
       </c>
       <c r="I8" s="4">
-        <v>188</v>
+        <v>562</v>
       </c>
       <c r="J8" s="4">
-        <v>124</v>
+        <v>463</v>
       </c>
       <c r="K8" s="4">
-        <v>78</v>
+        <v>246</v>
       </c>
       <c r="L8" s="4">
-        <v>3301</v>
+        <v>4201</v>
       </c>
       <c r="M8" s="4">
         <v>3467</v>
@@ -2119,10 +2234,10 @@
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="B9" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C9" s="4">
         <v>803</v>
@@ -2140,19 +2255,19 @@
         <v>454</v>
       </c>
       <c r="H9" s="4">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="I9" s="4">
-        <v>167</v>
+        <v>499</v>
       </c>
       <c r="J9" s="4">
-        <v>113</v>
+        <v>395</v>
       </c>
       <c r="K9" s="4">
-        <v>73</v>
+        <v>255</v>
       </c>
       <c r="L9" s="4">
-        <v>3039</v>
+        <v>3838</v>
       </c>
       <c r="M9" s="4">
         <v>3467</v>
@@ -2160,10 +2275,10 @@
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="B10" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C10" s="4">
         <v>722</v>
@@ -2184,16 +2299,16 @@
         <v>156</v>
       </c>
       <c r="I10" s="4">
-        <v>158</v>
+        <v>382</v>
       </c>
       <c r="J10" s="4">
-        <v>98</v>
+        <v>221</v>
       </c>
       <c r="K10" s="4">
-        <v>69</v>
+        <v>189</v>
       </c>
       <c r="L10" s="4">
-        <v>2729</v>
+        <v>3196</v>
       </c>
       <c r="M10" s="4">
         <v>3467</v>
@@ -2201,10 +2316,10 @@
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="B11" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C11" s="4">
         <v>673</v>
@@ -2225,16 +2340,16 @@
         <v>145</v>
       </c>
       <c r="I11" s="4">
-        <v>147</v>
+        <v>319</v>
       </c>
       <c r="J11" s="4">
-        <v>102</v>
+        <v>218</v>
       </c>
       <c r="K11" s="4">
-        <v>62</v>
+        <v>123</v>
       </c>
       <c r="L11" s="4">
-        <v>2536</v>
+        <v>2885</v>
       </c>
       <c r="M11" s="4">
         <v>3467</v>
@@ -2242,10 +2357,10 @@
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>59</v>
+        <v>69</v>
       </c>
       <c r="B12" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C12" s="4">
         <v>707</v>
@@ -2266,16 +2381,16 @@
         <v>147</v>
       </c>
       <c r="I12" s="4">
-        <v>157</v>
+        <v>357</v>
       </c>
       <c r="J12" s="4">
-        <v>104</v>
+        <v>272</v>
       </c>
       <c r="K12" s="4">
-        <v>64</v>
+        <v>162</v>
       </c>
       <c r="L12" s="4">
-        <v>2675</v>
+        <v>3140</v>
       </c>
       <c r="M12" s="4">
         <v>3467</v>
@@ -2283,10 +2398,10 @@
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="B13" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C13" s="4">
         <v>787</v>
@@ -2307,16 +2422,16 @@
         <v>164</v>
       </c>
       <c r="I13" s="4">
-        <v>174</v>
+        <v>546</v>
       </c>
       <c r="J13" s="4">
-        <v>119</v>
+        <v>398</v>
       </c>
       <c r="K13" s="4">
-        <v>81</v>
+        <v>285</v>
       </c>
       <c r="L13" s="4">
-        <v>3073</v>
+        <v>3928</v>
       </c>
       <c r="M13" s="4">
         <v>3467</v>
@@ -2324,10 +2439,10 @@
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="B14" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C14" s="4">
         <v>881</v>
@@ -2336,7 +2451,7 @@
         <v>291</v>
       </c>
       <c r="E14" s="4">
-        <v>622</v>
+        <v>633</v>
       </c>
       <c r="F14" s="4">
         <v>470</v>
@@ -2345,19 +2460,19 @@
         <v>495</v>
       </c>
       <c r="H14" s="4">
-        <v>188</v>
+        <v>340</v>
       </c>
       <c r="I14" s="4">
-        <v>192</v>
+        <v>696</v>
       </c>
       <c r="J14" s="4">
-        <v>122</v>
+        <v>465</v>
       </c>
       <c r="K14" s="4">
-        <v>86</v>
+        <v>334</v>
       </c>
       <c r="L14" s="4">
-        <v>3346</v>
+        <v>4604</v>
       </c>
       <c r="M14" s="4">
         <v>3467</v>
@@ -2365,10 +2480,10 @@
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>72</v>
+      </c>
+      <c r="B15" t="s">
         <v>62</v>
-      </c>
-      <c r="B15" t="s">
-        <v>52</v>
       </c>
       <c r="C15" s="4">
         <v>808</v>
@@ -2377,7 +2492,7 @@
         <v>281</v>
       </c>
       <c r="E15" s="4">
-        <v>558</v>
+        <v>582</v>
       </c>
       <c r="F15" s="4">
         <v>451</v>
@@ -2386,19 +2501,19 @@
         <v>456</v>
       </c>
       <c r="H15" s="4">
-        <v>171</v>
+        <v>284</v>
       </c>
       <c r="I15" s="4">
-        <v>182</v>
+        <v>565</v>
       </c>
       <c r="J15" s="4">
-        <v>117</v>
+        <v>399</v>
       </c>
       <c r="K15" s="4">
-        <v>79</v>
+        <v>260</v>
       </c>
       <c r="L15" s="4">
-        <v>3102</v>
+        <v>4086</v>
       </c>
       <c r="M15" s="4">
         <v>3467</v>
@@ -2406,10 +2521,10 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="B16" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C16" s="4">
         <v>647</v>
@@ -2430,16 +2545,16 @@
         <v>141</v>
       </c>
       <c r="I16" s="4">
-        <v>144</v>
+        <v>239</v>
       </c>
       <c r="J16" s="4">
-        <v>84</v>
+        <v>175</v>
       </c>
       <c r="K16" s="4">
-        <v>63</v>
+        <v>109</v>
       </c>
       <c r="L16" s="4">
-        <v>2520</v>
+        <v>2752</v>
       </c>
       <c r="M16" s="4">
         <v>3467</v>
@@ -2447,10 +2562,10 @@
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="B17" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C17" s="4">
         <v>745</v>
@@ -2471,16 +2586,16 @@
         <v>160</v>
       </c>
       <c r="I17" s="4">
-        <v>167</v>
+        <v>458</v>
       </c>
       <c r="J17" s="4">
-        <v>114</v>
+        <v>360</v>
       </c>
       <c r="K17" s="4">
-        <v>70</v>
+        <v>186</v>
       </c>
       <c r="L17" s="4">
-        <v>2907</v>
+        <v>3559</v>
       </c>
       <c r="M17" s="4">
         <v>3467</v>
@@ -2488,10 +2603,10 @@
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="B18" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C18" s="4">
         <v>819</v>
@@ -2512,16 +2627,16 @@
         <v>165</v>
       </c>
       <c r="I18" s="4">
-        <v>178</v>
+        <v>532</v>
       </c>
       <c r="J18" s="4">
-        <v>117</v>
+        <v>445</v>
       </c>
       <c r="K18" s="4">
-        <v>76</v>
+        <v>230</v>
       </c>
       <c r="L18" s="4">
-        <v>3071</v>
+        <v>3907</v>
       </c>
       <c r="M18" s="4">
         <v>3467</v>
@@ -2529,10 +2644,10 @@
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="B19" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C19" s="4">
         <v>812</v>
@@ -2553,16 +2668,16 @@
         <v>180</v>
       </c>
       <c r="I19" s="4">
-        <v>180</v>
+        <v>586</v>
       </c>
       <c r="J19" s="4">
-        <v>250</v>
+        <v>467</v>
       </c>
       <c r="K19" s="4">
-        <v>82</v>
+        <v>296</v>
       </c>
       <c r="L19" s="4">
-        <v>3335</v>
+        <v>4172</v>
       </c>
       <c r="M19" s="4">
         <v>3467</v>
@@ -2570,10 +2685,10 @@
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="B20" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C20" s="4">
         <v>795</v>
@@ -2594,16 +2709,16 @@
         <v>172</v>
       </c>
       <c r="I20" s="4">
-        <v>173</v>
+        <v>594</v>
       </c>
       <c r="J20" s="4">
-        <v>182</v>
+        <v>445</v>
       </c>
       <c r="K20" s="4">
-        <v>87</v>
+        <v>249</v>
       </c>
       <c r="L20" s="4">
-        <v>3133</v>
+        <v>3979</v>
       </c>
       <c r="M20" s="4">
         <v>3467</v>
@@ -2611,10 +2726,10 @@
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="B21" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C21" s="4">
         <v>743</v>
@@ -2635,16 +2750,16 @@
         <v>165</v>
       </c>
       <c r="I21" s="4">
-        <v>185</v>
+        <v>461</v>
       </c>
       <c r="J21" s="4">
-        <v>174</v>
+        <v>391</v>
       </c>
       <c r="K21" s="4">
-        <v>74</v>
+        <v>220</v>
       </c>
       <c r="L21" s="4">
-        <v>2997</v>
+        <v>3635</v>
       </c>
       <c r="M21" s="4">
         <v>3467</v>
@@ -2652,10 +2767,10 @@
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="B22" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C22" s="4">
         <v>689</v>
@@ -2676,16 +2791,16 @@
         <v>153</v>
       </c>
       <c r="I22" s="4">
-        <v>152</v>
+        <v>267</v>
       </c>
       <c r="J22" s="4">
-        <v>108</v>
+        <v>294</v>
       </c>
       <c r="K22" s="4">
-        <v>66</v>
+        <v>136</v>
       </c>
       <c r="L22" s="4">
-        <v>2663</v>
+        <v>3033</v>
       </c>
       <c r="M22" s="4">
         <v>3467</v>
@@ -2693,10 +2808,10 @@
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="B23" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C23" s="4">
         <v>655</v>
@@ -2717,16 +2832,16 @@
         <v>139</v>
       </c>
       <c r="I23" s="4">
-        <v>145</v>
+        <v>228</v>
       </c>
       <c r="J23" s="4">
-        <v>101</v>
+        <v>292</v>
       </c>
       <c r="K23" s="4">
-        <v>69</v>
+        <v>94</v>
       </c>
       <c r="L23" s="4">
-        <v>2539</v>
+        <v>2839</v>
       </c>
       <c r="M23" s="4">
         <v>3467</v>
@@ -2734,10 +2849,10 @@
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="B24" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C24" s="4">
         <v>687</v>
@@ -2758,16 +2873,16 @@
         <v>148</v>
       </c>
       <c r="I24" s="4">
-        <v>156</v>
+        <v>288</v>
       </c>
       <c r="J24" s="4">
-        <v>103</v>
+        <v>301</v>
       </c>
       <c r="K24" s="4">
-        <v>63</v>
+        <v>127</v>
       </c>
       <c r="L24" s="4">
-        <v>2619</v>
+        <v>3012</v>
       </c>
       <c r="M24" s="4">
         <v>3467</v>
@@ -2775,10 +2890,10 @@
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="B25" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C25" s="4">
         <v>798</v>
@@ -2799,16 +2914,16 @@
         <v>169</v>
       </c>
       <c r="I25" s="4">
-        <v>174</v>
+        <v>491</v>
       </c>
       <c r="J25" s="4">
-        <v>217</v>
+        <v>478</v>
       </c>
       <c r="K25" s="4">
-        <v>84</v>
+        <v>251</v>
       </c>
       <c r="L25" s="4">
-        <v>3159</v>
+        <v>3905</v>
       </c>
       <c r="M25" s="4">
         <v>3467</v>
@@ -2816,10 +2931,10 @@
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="B26" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C26" s="4">
         <v>835</v>
@@ -2837,19 +2952,19 @@
         <v>498</v>
       </c>
       <c r="H26" s="4">
-        <v>172</v>
+        <v>273</v>
       </c>
       <c r="I26" s="4">
-        <v>386</v>
+        <v>652</v>
       </c>
       <c r="J26" s="4">
-        <v>364</v>
+        <v>554</v>
       </c>
       <c r="K26" s="4">
-        <v>204</v>
+        <v>328</v>
       </c>
       <c r="L26" s="4">
-        <v>3846</v>
+        <v>4528</v>
       </c>
       <c r="M26" s="4">
         <v>3467</v>
@@ -2857,10 +2972,10 @@
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="B27" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C27" s="4">
         <v>820</v>
@@ -2878,19 +2993,19 @@
         <v>461</v>
       </c>
       <c r="H27" s="4">
-        <v>154</v>
+        <v>201</v>
       </c>
       <c r="I27" s="4">
-        <v>354</v>
+        <v>550</v>
       </c>
       <c r="J27" s="4">
-        <v>273</v>
+        <v>401</v>
       </c>
       <c r="K27" s="4">
-        <v>134</v>
+        <v>257</v>
       </c>
       <c r="L27" s="4">
-        <v>3491</v>
+        <v>3984</v>
       </c>
       <c r="M27" s="4">
         <v>3467</v>
@@ -2898,10 +3013,10 @@
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="B28" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C28" s="4">
         <v>641</v>
@@ -2922,16 +3037,16 @@
         <v>133</v>
       </c>
       <c r="I28" s="4">
-        <v>141</v>
+        <v>197</v>
       </c>
       <c r="J28" s="4">
-        <v>105</v>
+        <v>224</v>
       </c>
       <c r="K28" s="4">
-        <v>64</v>
+        <v>123</v>
       </c>
       <c r="L28" s="4">
-        <v>2473</v>
+        <v>2708</v>
       </c>
       <c r="M28" s="4">
         <v>3467</v>
@@ -2939,10 +3054,10 @@
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="B29" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C29" s="4">
         <v>767</v>
@@ -2963,16 +3078,16 @@
         <v>157</v>
       </c>
       <c r="I29" s="4">
-        <v>192</v>
+        <v>385</v>
       </c>
       <c r="J29" s="4">
-        <v>242</v>
+        <v>332</v>
       </c>
       <c r="K29" s="4">
-        <v>97</v>
+        <v>209</v>
       </c>
       <c r="L29" s="4">
-        <v>3071</v>
+        <v>3466</v>
       </c>
       <c r="M29" s="4">
         <v>3467</v>
@@ -2980,10 +3095,10 @@
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="B30" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C30" s="4">
         <v>765</v>
@@ -3004,16 +3119,16 @@
         <v>169</v>
       </c>
       <c r="I30" s="4">
-        <v>343</v>
+        <v>457</v>
       </c>
       <c r="J30" s="4">
-        <v>373</v>
+        <v>417</v>
       </c>
       <c r="K30" s="4">
-        <v>179</v>
+        <v>246</v>
       </c>
       <c r="L30" s="4">
-        <v>3559</v>
+        <v>3785</v>
       </c>
       <c r="M30" s="4">
         <v>3467</v>
@@ -3021,10 +3136,10 @@
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="B31" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C31" s="4">
         <v>794</v>
@@ -3045,16 +3160,16 @@
         <v>176</v>
       </c>
       <c r="I31" s="4">
-        <v>432</v>
+        <v>498</v>
       </c>
       <c r="J31" s="4">
-        <v>393</v>
+        <v>469</v>
       </c>
       <c r="K31" s="4">
-        <v>189</v>
+        <v>247</v>
       </c>
       <c r="L31" s="4">
-        <v>3788</v>
+        <v>3987</v>
       </c>
       <c r="M31" s="4">
         <v>3467</v>
@@ -3062,10 +3177,10 @@
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="B32" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C32" s="4">
         <v>760</v>
@@ -3086,16 +3201,16 @@
         <v>159</v>
       </c>
       <c r="I32" s="4">
-        <v>417</v>
+        <v>496</v>
       </c>
       <c r="J32" s="4">
-        <v>408</v>
+        <v>393</v>
       </c>
       <c r="K32" s="4">
-        <v>226</v>
+        <v>264</v>
       </c>
       <c r="L32" s="4">
-        <v>3664</v>
+        <v>3767</v>
       </c>
       <c r="M32" s="4">
         <v>3467</v>
@@ -3103,10 +3218,10 @@
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B33" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C33" s="4">
         <v>734</v>
@@ -3127,16 +3242,16 @@
         <v>153</v>
       </c>
       <c r="I33" s="4">
-        <v>374</v>
+        <v>402</v>
       </c>
       <c r="J33" s="4">
-        <v>327</v>
+        <v>322</v>
       </c>
       <c r="K33" s="4">
-        <v>129</v>
+        <v>163</v>
       </c>
       <c r="L33" s="4">
-        <v>3335</v>
+        <v>3392</v>
       </c>
       <c r="M33" s="4">
         <v>3467</v>
@@ -3144,10 +3259,10 @@
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="B34" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C34" s="4">
         <v>676</v>
@@ -3168,16 +3283,16 @@
         <v>144</v>
       </c>
       <c r="I34" s="4">
-        <v>287</v>
+        <v>304</v>
       </c>
       <c r="J34" s="4">
-        <v>278</v>
+        <v>237</v>
       </c>
       <c r="K34" s="4">
-        <v>103</v>
+        <v>149</v>
       </c>
       <c r="L34" s="4">
-        <v>2954</v>
+        <v>2975</v>
       </c>
       <c r="M34" s="4">
         <v>3467</v>
@@ -3185,10 +3300,10 @@
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="B35" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C35" s="4">
         <v>621</v>
@@ -3209,16 +3324,16 @@
         <v>130</v>
       </c>
       <c r="I35" s="4">
-        <v>175</v>
+        <v>188</v>
       </c>
       <c r="J35" s="4">
-        <v>231</v>
+        <v>173</v>
       </c>
       <c r="K35" s="4">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="L35" s="4">
-        <v>2609</v>
+        <v>2544</v>
       </c>
       <c r="M35" s="4">
         <v>3467</v>
@@ -3226,10 +3341,10 @@
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="B36" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C36" s="4">
         <v>638</v>
@@ -3250,16 +3365,16 @@
         <v>136</v>
       </c>
       <c r="I36" s="4">
-        <v>225</v>
+        <v>171</v>
       </c>
       <c r="J36" s="4">
-        <v>279</v>
+        <v>224</v>
       </c>
       <c r="K36" s="4">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="L36" s="4">
-        <v>2848</v>
+        <v>2727</v>
       </c>
       <c r="M36" s="4">
         <v>3467</v>
@@ -3267,10 +3382,10 @@
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="B37" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C37" s="4">
         <v>767</v>
@@ -3291,16 +3406,16 @@
         <v>160</v>
       </c>
       <c r="I37" s="4">
-        <v>499</v>
+        <v>473</v>
       </c>
       <c r="J37" s="4">
-        <v>458</v>
+        <v>379</v>
       </c>
       <c r="K37" s="4">
-        <v>222</v>
+        <v>228</v>
       </c>
       <c r="L37" s="4">
-        <v>3800</v>
+        <v>3701</v>
       </c>
       <c r="M37" s="4">
         <v>3467</v>
@@ -3308,10 +3423,10 @@
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="B38" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="C38" s="4">
         <v>835</v>
@@ -3320,28 +3435,28 @@
         <v>290</v>
       </c>
       <c r="E38" s="4">
-        <v>1123</v>
+        <v>926</v>
       </c>
       <c r="F38" s="4">
-        <v>793</v>
+        <v>565</v>
       </c>
       <c r="G38" s="4">
-        <v>775</v>
+        <v>599</v>
       </c>
       <c r="H38" s="4">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="I38" s="4">
-        <v>663</v>
+        <v>666</v>
       </c>
       <c r="J38" s="4">
-        <v>532</v>
+        <v>493</v>
       </c>
       <c r="K38" s="4">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="L38" s="4">
-        <v>5668</v>
+        <v>5032</v>
       </c>
       <c r="M38" s="4">
         <v>3467</v>
@@ -3349,10 +3464,10 @@
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="B39" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="C39" s="4">
         <v>775</v>
@@ -3361,28 +3476,28 @@
         <v>269</v>
       </c>
       <c r="E39" s="4">
-        <v>837</v>
+        <v>680</v>
       </c>
       <c r="F39" s="4">
-        <v>562</v>
+        <v>428</v>
       </c>
       <c r="G39" s="4">
-        <v>569</v>
+        <v>448</v>
       </c>
       <c r="H39" s="4">
-        <v>248</v>
+        <v>257</v>
       </c>
       <c r="I39" s="4">
-        <v>561</v>
+        <v>575</v>
       </c>
       <c r="J39" s="4">
-        <v>461</v>
+        <v>433</v>
       </c>
       <c r="K39" s="4">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="L39" s="4">
-        <v>4563</v>
+        <v>4149</v>
       </c>
       <c r="M39" s="4">
         <v>3467</v>
@@ -3390,10 +3505,10 @@
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="B40" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="C40" s="4">
         <v>627</v>
@@ -3414,16 +3529,16 @@
         <v>133</v>
       </c>
       <c r="I40" s="4">
-        <v>281</v>
+        <v>303</v>
       </c>
       <c r="J40" s="4">
-        <v>268</v>
+        <v>250</v>
       </c>
       <c r="K40" s="4">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="L40" s="4">
-        <v>2834</v>
+        <v>2845</v>
       </c>
       <c r="M40" s="4">
         <v>3467</v>
@@ -3431,10 +3546,10 @@
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="B41" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="C41" s="4">
         <v>723</v>
@@ -3443,28 +3558,28 @@
         <v>251</v>
       </c>
       <c r="E41" s="4">
-        <v>674</v>
+        <v>584</v>
       </c>
       <c r="F41" s="4">
-        <v>449</v>
+        <v>399</v>
       </c>
       <c r="G41" s="4">
-        <v>461</v>
+        <v>417</v>
       </c>
       <c r="H41" s="4">
-        <v>202</v>
+        <v>214</v>
       </c>
       <c r="I41" s="4">
-        <v>452</v>
+        <v>476</v>
       </c>
       <c r="J41" s="4">
-        <v>366</v>
+        <v>357</v>
       </c>
       <c r="K41" s="4">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="L41" s="4">
-        <v>3806</v>
+        <v>3658</v>
       </c>
       <c r="M41" s="4">
         <v>3467</v>
@@ -3472,40 +3587,40 @@
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="B42" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="C42" s="4">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="D42" s="4">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E42" s="4">
-        <v>883</v>
+        <v>803</v>
       </c>
       <c r="F42" s="4">
-        <v>619</v>
+        <v>483</v>
       </c>
       <c r="G42" s="4">
-        <v>607</v>
+        <v>505</v>
       </c>
       <c r="H42" s="4">
-        <v>258</v>
+        <v>270</v>
       </c>
       <c r="I42" s="4">
-        <v>516</v>
+        <v>543</v>
       </c>
       <c r="J42" s="4">
-        <v>408</v>
+        <v>404</v>
       </c>
       <c r="K42" s="4">
-        <v>259</v>
+        <v>270</v>
       </c>
       <c r="L42" s="4">
-        <v>4562</v>
+        <v>4289</v>
       </c>
       <c r="M42" s="4">
         <v>3467</v>
@@ -3513,10 +3628,10 @@
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="B43" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="C43" s="4">
         <v>785</v>
@@ -3525,28 +3640,28 @@
         <v>273</v>
       </c>
       <c r="E43" s="4">
-        <v>1129</v>
+        <v>1054</v>
       </c>
       <c r="F43" s="4">
-        <v>819</v>
+        <v>684</v>
       </c>
       <c r="G43" s="4">
-        <v>779</v>
+        <v>677</v>
       </c>
       <c r="H43" s="4">
-        <v>325</v>
+        <v>336</v>
       </c>
       <c r="I43" s="4">
-        <v>594</v>
+        <v>622</v>
       </c>
       <c r="J43" s="4">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="K43" s="4">
-        <v>295</v>
+        <v>308</v>
       </c>
       <c r="L43" s="4">
-        <v>5458</v>
+        <v>5196</v>
       </c>
       <c r="M43" s="4">
         <v>3467</v>
@@ -3554,40 +3669,40 @@
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="B44" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="C44" s="4">
         <v>762</v>
       </c>
       <c r="D44" s="4">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="E44" s="4">
-        <v>1067</v>
+        <v>992</v>
       </c>
       <c r="F44" s="4">
-        <v>772</v>
+        <v>634</v>
       </c>
       <c r="G44" s="4">
-        <v>735</v>
+        <v>630</v>
       </c>
       <c r="H44" s="4">
-        <v>308</v>
+        <v>316</v>
       </c>
       <c r="I44" s="4">
-        <v>569</v>
+        <v>597</v>
       </c>
       <c r="J44" s="4">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="K44" s="4">
-        <v>283</v>
+        <v>296</v>
       </c>
       <c r="L44" s="4">
-        <v>5201</v>
+        <v>4932</v>
       </c>
       <c r="M44" s="4">
         <v>3467</v>
@@ -3595,10 +3710,10 @@
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="B45" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="C45" s="4">
         <v>710</v>
@@ -3607,28 +3722,28 @@
         <v>246</v>
       </c>
       <c r="E45" s="4">
-        <v>853</v>
+        <v>774</v>
       </c>
       <c r="F45" s="4">
-        <v>601</v>
+        <v>457</v>
       </c>
       <c r="G45" s="4">
-        <v>584</v>
+        <v>474</v>
       </c>
       <c r="H45" s="4">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="I45" s="4">
-        <v>494</v>
+        <v>520</v>
       </c>
       <c r="J45" s="4">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="K45" s="4">
-        <v>248</v>
+        <v>261</v>
       </c>
       <c r="L45" s="4">
-        <v>4376</v>
+        <v>4087</v>
       </c>
       <c r="M45" s="4">
         <v>3467</v>
@@ -3636,10 +3751,10 @@
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="B46" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="C46" s="4">
         <v>644</v>
@@ -3648,28 +3763,28 @@
         <v>224</v>
       </c>
       <c r="E46" s="4">
-        <v>565</v>
+        <v>478</v>
       </c>
       <c r="F46" s="4">
-        <v>370</v>
+        <v>355</v>
       </c>
       <c r="G46" s="4">
-        <v>381</v>
+        <v>372</v>
       </c>
       <c r="H46" s="4">
         <v>172</v>
       </c>
       <c r="I46" s="4">
-        <v>392</v>
+        <v>416</v>
       </c>
       <c r="J46" s="4">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="K46" s="4">
-        <v>201</v>
+        <v>213</v>
       </c>
       <c r="L46" s="4">
-        <v>3268</v>
+        <v>3196</v>
       </c>
       <c r="M46" s="4">
         <v>3467</v>
@@ -3677,10 +3792,10 @@
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="B47" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="C47" s="4">
         <v>607</v>
@@ -3698,19 +3813,19 @@
         <v>350</v>
       </c>
       <c r="H47" s="4">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="I47" s="4">
-        <v>342</v>
+        <v>364</v>
       </c>
       <c r="J47" s="4">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="K47" s="4">
-        <v>178</v>
+        <v>189</v>
       </c>
       <c r="L47" s="4">
-        <v>2872</v>
+        <v>2902</v>
       </c>
       <c r="M47" s="4">
         <v>3467</v>
@@ -3718,10 +3833,10 @@
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
+        <v>106</v>
+      </c>
+      <c r="B48" t="s">
         <v>96</v>
-      </c>
-      <c r="B48" t="s">
-        <v>86</v>
       </c>
       <c r="C48" s="4">
         <v>634</v>
@@ -3730,28 +3845,28 @@
         <v>220</v>
       </c>
       <c r="E48" s="4">
-        <v>628</v>
+        <v>513</v>
       </c>
       <c r="F48" s="4">
-        <v>423</v>
+        <v>350</v>
       </c>
       <c r="G48" s="4">
-        <v>423</v>
+        <v>366</v>
       </c>
       <c r="H48" s="4">
-        <v>189</v>
+        <v>179</v>
       </c>
       <c r="I48" s="4">
-        <v>405</v>
+        <v>422</v>
       </c>
       <c r="J48" s="4">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="K48" s="4">
-        <v>206</v>
+        <v>216</v>
       </c>
       <c r="L48" s="4">
-        <v>3454</v>
+        <v>3227</v>
       </c>
       <c r="M48" s="4">
         <v>3467</v>
@@ -3759,40 +3874,40 @@
     </row>
     <row r="49" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="B49" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="C49" s="4">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="D49" s="4">
         <v>257</v>
       </c>
       <c r="E49" s="4">
-        <v>1239</v>
+        <v>1108</v>
       </c>
       <c r="F49" s="4">
-        <v>919</v>
+        <v>725</v>
       </c>
       <c r="G49" s="4">
-        <v>851</v>
+        <v>698</v>
       </c>
       <c r="H49" s="4">
-        <v>354</v>
+        <v>338</v>
       </c>
       <c r="I49" s="4">
-        <v>605</v>
+        <v>618</v>
       </c>
       <c r="J49" s="4">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="K49" s="4">
-        <v>299</v>
+        <v>307</v>
       </c>
       <c r="L49" s="4">
-        <v>5725</v>
+        <v>5250</v>
       </c>
       <c r="M49" s="4">
         <v>3467</v>
@@ -3800,10 +3915,10 @@
     </row>
     <row r="50" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="B50" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="C50" s="4">
         <v>809</v>
@@ -3812,28 +3927,28 @@
         <v>281</v>
       </c>
       <c r="E50" s="4">
-        <v>1660</v>
+        <v>1510</v>
       </c>
       <c r="F50" s="4">
-        <v>1261</v>
+        <v>1050</v>
       </c>
       <c r="G50" s="4">
-        <v>1146</v>
+        <v>980</v>
       </c>
       <c r="H50" s="4">
-        <v>468</v>
+        <v>446</v>
       </c>
       <c r="I50" s="4">
-        <v>743</v>
+        <v>750</v>
       </c>
       <c r="J50" s="4">
-        <v>552</v>
+        <v>549</v>
       </c>
       <c r="K50" s="4">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="L50" s="4">
-        <v>7283</v>
+        <v>6744</v>
       </c>
       <c r="M50" s="4">
         <v>3467</v>
@@ -3841,40 +3956,40 @@
     </row>
     <row r="51" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="B51" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="C51" s="4">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="D51" s="4">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E51" s="4">
-        <v>1405</v>
+        <v>1234</v>
       </c>
       <c r="F51" s="4">
-        <v>1058</v>
+        <v>829</v>
       </c>
       <c r="G51" s="4">
-        <v>967</v>
+        <v>785</v>
       </c>
       <c r="H51" s="4">
-        <v>398</v>
+        <v>369</v>
       </c>
       <c r="I51" s="4">
-        <v>653</v>
+        <v>655</v>
       </c>
       <c r="J51" s="4">
-        <v>490</v>
+        <v>485</v>
       </c>
       <c r="K51" s="4">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="L51" s="4">
-        <v>6303</v>
+        <v>5693</v>
       </c>
       <c r="M51" s="4">
         <v>3467</v>
@@ -3882,40 +3997,40 @@
     </row>
     <row r="52" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="B52" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="C52" s="4">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="D52" s="4">
         <v>211</v>
       </c>
       <c r="E52" s="4">
-        <v>702</v>
+        <v>509</v>
       </c>
       <c r="F52" s="4">
-        <v>491</v>
+        <v>335</v>
       </c>
       <c r="G52" s="4">
-        <v>474</v>
+        <v>351</v>
       </c>
       <c r="H52" s="4">
-        <v>208</v>
+        <v>172</v>
       </c>
       <c r="I52" s="4">
-        <v>415</v>
+        <v>411</v>
       </c>
       <c r="J52" s="4">
-        <v>329</v>
+        <v>321</v>
       </c>
       <c r="K52" s="4">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="L52" s="4">
-        <v>3647</v>
+        <v>3129</v>
       </c>
       <c r="M52" s="4">
         <v>3467</v>
@@ -3923,7 +4038,7 @@
     </row>
     <row r="54" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A54" s="7" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="C54" s="4">
         <v>9701</v>
@@ -3932,7 +4047,7 @@
         <v>3325</v>
       </c>
       <c r="E54" s="4">
-        <v>6607</v>
+        <v>6641</v>
       </c>
       <c r="F54" s="4">
         <v>5169</v>
@@ -3941,24 +4056,24 @@
         <v>5335</v>
       </c>
       <c r="H54" s="4">
-        <v>2009</v>
+        <v>2567</v>
       </c>
       <c r="I54" s="4">
-        <v>2056</v>
+        <v>6008</v>
       </c>
       <c r="J54" s="4">
-        <v>1342</v>
+        <v>4296</v>
       </c>
       <c r="K54" s="4">
-        <v>875</v>
-      </c>
-      <c r="L54" s="14">
-        <v>36419</v>
+        <v>2812</v>
+      </c>
+      <c r="L54" s="10">
+        <v>45854</v>
       </c>
     </row>
     <row r="55" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A55" s="7" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="C55" s="4">
         <v>9040</v>
@@ -3976,24 +4091,24 @@
         <v>5209</v>
       </c>
       <c r="H55" s="4">
-        <v>1910</v>
+        <v>2058</v>
       </c>
       <c r="I55" s="4">
-        <v>2390</v>
+        <v>5303</v>
       </c>
       <c r="J55" s="4">
-        <v>2108</v>
+        <v>4650</v>
       </c>
       <c r="K55" s="4">
-        <v>1071</v>
-      </c>
-      <c r="L55" s="14">
-        <v>36233</v>
+        <v>2497</v>
+      </c>
+      <c r="L55" s="10">
+        <v>43261</v>
       </c>
     </row>
     <row r="56" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A56" s="7" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="C56" s="4">
         <v>6521</v>
@@ -4014,16 +4129,16 @@
         <v>1385</v>
       </c>
       <c r="I56" s="4">
-        <v>2945</v>
+        <v>3375</v>
       </c>
       <c r="J56" s="4">
-        <v>2989</v>
+        <v>2946</v>
       </c>
       <c r="K56" s="4">
-        <v>1368</v>
-      </c>
-      <c r="L56" s="14">
-        <v>29626</v>
+        <v>1697</v>
+      </c>
+      <c r="L56" s="10">
+        <v>30343</v>
       </c>
     </row>
   </sheetData>
@@ -4045,114 +4160,114 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
-        <v>106</v>
+      <c r="A2" s="11" t="s">
+        <v>116</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="15" t="s">
-        <v>108</v>
+      <c r="A3" s="11" t="s">
+        <v>118</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="15" t="s">
-        <v>110</v>
+      <c r="A4" s="11" t="s">
+        <v>120</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="15" t="s">
-        <v>112</v>
+      <c r="A5" s="11" t="s">
+        <v>122</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="15" t="s">
-        <v>114</v>
+      <c r="A6" s="11" t="s">
+        <v>124</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="15" t="s">
-        <v>116</v>
+        <v>125</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="105" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="11" t="s">
+        <v>126</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="15" t="s">
-        <v>118</v>
+      <c r="A8" s="11" t="s">
+        <v>128</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="15" t="s">
-        <v>120</v>
+      <c r="A9" s="11" t="s">
+        <v>130</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>121</v>
+        <v>131</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="15" t="s">
-        <v>122</v>
+      <c r="A10" s="11" t="s">
+        <v>132</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="15" t="s">
-        <v>124</v>
+      <c r="A11" s="11" t="s">
+        <v>134</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="15" t="s">
-        <v>126</v>
+      <c r="A12" s="11" t="s">
+        <v>136</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>127</v>
+        <v>137</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="15" t="s">
-        <v>128</v>
+      <c r="A13" s="11" t="s">
+        <v>138</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>129</v>
+        <v>139</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="15" t="s">
-        <v>130</v>
+      <c r="A14" s="11" t="s">
+        <v>140</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>131</v>
+        <v>141</v>
       </c>
     </row>
   </sheetData>

</xml_diff>